<commit_message>
premiere version de la copie à deployer sur le serveur de la CAE
</commit_message>
<xml_diff>
--- a/OneDrive - GOUVCI/DCSARD/Action_Regionale/App/dashbord-Anstat-version_V2_atelier/dashbord-Anstat-version_V2_atelier/static/data/publications2.xlsx
+++ b/OneDrive - GOUVCI/DCSARD/Action_Regionale/App/dashbord-Anstat-version_V2_atelier/dashbord-Anstat-version_V2_atelier/static/data/publications2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive - GOUVCI\DCSARD\Action_Regionale\App\dashbord-Anstat-version_V2_atelier\dashbord-Anstat-version_V2_atelier\static\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEA0DDA5-CE53-4D65-BE81-BC81E54BD52B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{778F3F38-4B58-4AFB-93FA-DC1F4E7DB84C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -363,6 +363,7 @@
     <col min="2" max="3" width="12.6328125" customWidth="1"/>
     <col min="4" max="4" width="45.26953125" customWidth="1"/>
     <col min="5" max="6" width="12.6328125" customWidth="1"/>
+    <col min="7" max="7" width="30.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>